<commit_message>
Refresh SDTM CT to 2026-09-25 (NCI EVS)
- SDTM CT pin 2026-03-27 -> 2026-09-25 in both download copies
  (sdtm-test-codes, cosmos-bc-dss); NCIt Thesaurus FLAT and CUI map
  refreshed alongside - the April copy lacked most codes new to this CT.
  Previous inputs kept in downloads/_prev_2026-03-27/ (gitignored)
- Version strings updated in five notebook README cells, CLAUDE.md,
  README.md, sdtm-findings-graph/README.md; COSMoS version there
  corrected from 2026-Q1 to 2026-07-14
- Re-run: sdtm-test-codes (4), cosmos-graph 20/30/40/50/51,
  consumer-bases 10/20/30, sdtm-findings-graph (3), link-semantics (2);
  pipeline code unchanged, COSMoS 2026-07-14 unchanged
- New unresolved concept ID C181502 (GPBAEST, retired in this CT);
  r18 PROCEDUR/METHOD value-list members still absent from CT
- docs/Changes_2026-09.md: release note

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSD59mvcqpub3JwR483ah8
</commit_message>
<xml_diff>
--- a/consumer-bases/interim/PR_DSS_Reachability.xlsx
+++ b/consumer-bases/interim/PR_DSS_Reachability.xlsx
@@ -484,7 +484,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-08-23 19:06</t>
+          <t>Generated: 2026-09-30 18:20</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Sources: COSMoS public exports + NCI EVS CT package 2026-03-27.</t>
+          <t>Sources: COSMoS public exports + NCI EVS CT package 2026-09-25.</t>
         </is>
       </c>
     </row>

</xml_diff>